<commit_message>
grille commerciale v1.2 : une prime unique par garage, prime de fidélité supprimée (documents + espace éditeur)
</commit_message>
<xml_diff>
--- a/docs/pack-commercial/commerciaux/SIMULATEUR-COMMISSIONS.xlsx
+++ b/docs/pack-commercial/commerciaux/SIMULATEUR-COMMISSIONS.xlsx
@@ -36,7 +36,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Part des garages signés toujours actifs (et à jour) au 6e mois — conditionne la prime de fidélité.</t>
+          <t xml:space="preserve">Ne sert que si une prime de fidélité est réintroduite (colonne E).</t>
         </r>
       </text>
     </comment>
@@ -128,7 +128,7 @@
     <t xml:space="preserve">Prime de signature</t>
   </si>
   <si>
-    <t xml:space="preserve">Prime de fidélité (M6)</t>
+    <t xml:space="preserve">Prime de fidélité (0 en v1.2)</t>
   </si>
   <si>
     <t xml:space="preserve">Bonus engagement 12 mois</t>
@@ -191,13 +191,13 @@
     <t xml:space="preserve">Palier 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Source des prix et de la rétrocession : NOTE-STRATEGIE-TARIFAIRE et IDEAFORMA_modele_rentabilite.xlsx (docs/pack-commercial). Commissions : grille apporteurs v1.1 du 25/08/2026 (−15 % sur la v1.0).</t>
+    <t xml:space="preserve">Source des prix et de la rétrocession : NOTE-STRATEGIE-TARIFAIRE et IDEAFORMA_modele_rentabilite.xlsx (docs/pack-commercial). Commissions : grille apporteurs v1.2 du 25/08/2026 (une prime unique par garage, prime de fidélité supprimée).</t>
   </si>
   <si>
     <t xml:space="preserve">Ce que gagne le commercial selon son rythme</t>
   </si>
   <si>
-    <t xml:space="preserve">Saisissez vos signatures mensuelles par formule (jaune). Les montants perçus tiennent compte des délais de paiement (Paramètres).</t>
+    <t xml:space="preserve">Saisissez vos signatures mensuelles par formule (jaune). Grille v1.2 : une prime par garage signé, acquise à la 2e mensualité payée ; les montants perçus tiennent compte de ce délai (Paramètres).</t>
   </si>
   <si>
     <t xml:space="preserve">Signatures par mois</t>
@@ -1055,7 +1055,7 @@
         <v>130</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="F7" s="6" t="n">
         <v>40</v>
@@ -1083,7 +1083,7 @@
         <v>415</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>210</v>
+        <v>0</v>
       </c>
       <c r="F8" s="6" t="n">
         <v>85</v>
@@ -1111,7 +1111,7 @@
         <v>730</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>365</v>
+        <v>0</v>
       </c>
       <c r="F9" s="6" t="n">
         <v>85</v>
@@ -1139,7 +1139,7 @@
         <v>1335</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>665</v>
+        <v>0</v>
       </c>
       <c r="F10" s="6" t="n">
         <v>85</v>
@@ -1446,15 +1446,15 @@
       </c>
       <c r="B11" s="9" t="n">
         <f aca="false">B$5*Paramètres!$E$7*Paramètres!$G$13</f>
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="C11" s="9" t="n">
         <f aca="false">C$5*Paramètres!$E$8*Paramètres!$G$13</f>
-        <v>357</v>
+        <v>0</v>
       </c>
       <c r="D11" s="9" t="n">
         <f aca="false">D$5*Paramètres!$E$9*Paramètres!$G$13</f>
-        <v>310.25</v>
+        <v>0</v>
       </c>
       <c r="E11" s="9" t="n">
         <f aca="false">E$5*Paramètres!$E$10*Paramètres!$G$13</f>
@@ -1462,7 +1462,7 @@
       </c>
       <c r="F11" s="16" t="n">
         <f aca="false">SUM(B11:E11)</f>
-        <v>701.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1471,15 +1471,15 @@
       </c>
       <c r="B12" s="17" t="n">
         <f aca="false">SUM(B9:B11)</f>
-        <v>188</v>
+        <v>154</v>
       </c>
       <c r="C12" s="17" t="n">
         <f aca="false">SUM(C9:C11)</f>
-        <v>1289</v>
+        <v>932</v>
       </c>
       <c r="D12" s="17" t="n">
         <f aca="false">SUM(D9:D11)</f>
-        <v>1091.25</v>
+        <v>781</v>
       </c>
       <c r="E12" s="17" t="n">
         <f aca="false">SUM(E9:E11)</f>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="F12" s="17" t="n">
         <f aca="false">SUM(F9:F11)</f>
-        <v>2568.25</v>
+        <v>1867</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1711,7 +1711,7 @@
       </c>
       <c r="D23" s="9" t="n">
         <f aca="false">IF(A23&gt;Paramètres!$G$18,$F$11,0)</f>
-        <v>701.25</v>
+        <v>0</v>
       </c>
       <c r="E23" s="9" t="n">
         <f aca="false">IF(MOD(A23,3)=0,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$23,Paramètres!$C$23,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$22,Paramètres!$C$22,0)),0)</f>
@@ -1719,11 +1719,11 @@
       </c>
       <c r="F23" s="16" t="n">
         <f aca="false">C23+D23+E23</f>
-        <v>2568.25</v>
+        <v>1867</v>
       </c>
       <c r="G23" s="9" t="n">
         <f aca="false">SUM($F$17:F23)</f>
-        <v>10546.25</v>
+        <v>9845</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="D24" s="9" t="n">
         <f aca="false">IF(A24&gt;Paramètres!$G$18,$F$11,0)</f>
-        <v>701.25</v>
+        <v>0</v>
       </c>
       <c r="E24" s="9" t="n">
         <f aca="false">IF(MOD(A24,3)=0,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$23,Paramètres!$C$23,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$22,Paramètres!$C$22,0)),0)</f>
@@ -1748,11 +1748,11 @@
       </c>
       <c r="F24" s="16" t="n">
         <f aca="false">C24+D24+E24</f>
-        <v>2568.25</v>
+        <v>1867</v>
       </c>
       <c r="G24" s="9" t="n">
         <f aca="false">SUM($F$17:F24)</f>
-        <v>13114.5</v>
+        <v>11712</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1769,7 +1769,7 @@
       </c>
       <c r="D25" s="9" t="n">
         <f aca="false">IF(A25&gt;Paramètres!$G$18,$F$11,0)</f>
-        <v>701.25</v>
+        <v>0</v>
       </c>
       <c r="E25" s="9" t="n">
         <f aca="false">IF(MOD(A25,3)=0,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$23,Paramètres!$C$23,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$22,Paramètres!$C$22,0)),0)</f>
@@ -1777,11 +1777,11 @@
       </c>
       <c r="F25" s="16" t="n">
         <f aca="false">C25+D25+E25</f>
-        <v>2823.25</v>
+        <v>2122</v>
       </c>
       <c r="G25" s="9" t="n">
         <f aca="false">SUM($F$17:F25)</f>
-        <v>15937.75</v>
+        <v>13834</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="D26" s="9" t="n">
         <f aca="false">IF(A26&gt;Paramètres!$G$18,$F$11,0)</f>
-        <v>701.25</v>
+        <v>0</v>
       </c>
       <c r="E26" s="9" t="n">
         <f aca="false">IF(MOD(A26,3)=0,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$23,Paramètres!$C$23,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$22,Paramètres!$C$22,0)),0)</f>
@@ -1806,11 +1806,11 @@
       </c>
       <c r="F26" s="16" t="n">
         <f aca="false">C26+D26+E26</f>
-        <v>2568.25</v>
+        <v>1867</v>
       </c>
       <c r="G26" s="9" t="n">
         <f aca="false">SUM($F$17:F26)</f>
-        <v>18506</v>
+        <v>15701</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1827,7 +1827,7 @@
       </c>
       <c r="D27" s="9" t="n">
         <f aca="false">IF(A27&gt;Paramètres!$G$18,$F$11,0)</f>
-        <v>701.25</v>
+        <v>0</v>
       </c>
       <c r="E27" s="9" t="n">
         <f aca="false">IF(MOD(A27,3)=0,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$23,Paramètres!$C$23,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$22,Paramètres!$C$22,0)),0)</f>
@@ -1835,11 +1835,11 @@
       </c>
       <c r="F27" s="16" t="n">
         <f aca="false">C27+D27+E27</f>
-        <v>2568.25</v>
+        <v>1867</v>
       </c>
       <c r="G27" s="9" t="n">
         <f aca="false">SUM($F$17:F27)</f>
-        <v>21074.25</v>
+        <v>17568</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="D28" s="9" t="n">
         <f aca="false">IF(A28&gt;Paramètres!$G$18,$F$11,0)</f>
-        <v>701.25</v>
+        <v>0</v>
       </c>
       <c r="E28" s="9" t="n">
         <f aca="false">IF(MOD(A28,3)=0,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$23,Paramètres!$C$23,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$22,Paramètres!$C$22,0)),0)</f>
@@ -1864,11 +1864,11 @@
       </c>
       <c r="F28" s="16" t="n">
         <f aca="false">C28+D28+E28</f>
-        <v>2823.25</v>
+        <v>2122</v>
       </c>
       <c r="G28" s="9" t="n">
         <f aca="false">SUM($F$17:F28)</f>
-        <v>23897.5</v>
+        <v>19690</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="D29" s="9" t="n">
         <f aca="false">IF(A29&gt;Paramètres!$G$18,$F$11,0)</f>
-        <v>701.25</v>
+        <v>0</v>
       </c>
       <c r="E29" s="9" t="n">
         <f aca="false">IF(MOD(A29,3)=0,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$23,Paramètres!$C$23,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$22,Paramètres!$C$22,0)),0)</f>
@@ -1893,11 +1893,11 @@
       </c>
       <c r="F29" s="16" t="n">
         <f aca="false">C29+D29+E29</f>
-        <v>2568.25</v>
+        <v>1867</v>
       </c>
       <c r="G29" s="9" t="n">
         <f aca="false">SUM($F$17:F29)</f>
-        <v>26465.75</v>
+        <v>21557</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="D30" s="9" t="n">
         <f aca="false">IF(A30&gt;Paramètres!$G$18,$F$11,0)</f>
-        <v>701.25</v>
+        <v>0</v>
       </c>
       <c r="E30" s="9" t="n">
         <f aca="false">IF(MOD(A30,3)=0,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$23,Paramètres!$C$23,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$22,Paramètres!$C$22,0)),0)</f>
@@ -1922,11 +1922,11 @@
       </c>
       <c r="F30" s="16" t="n">
         <f aca="false">C30+D30+E30</f>
-        <v>2568.25</v>
+        <v>1867</v>
       </c>
       <c r="G30" s="9" t="n">
         <f aca="false">SUM($F$17:F30)</f>
-        <v>29034</v>
+        <v>23424</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="D31" s="9" t="n">
         <f aca="false">IF(A31&gt;Paramètres!$G$18,$F$11,0)</f>
-        <v>701.25</v>
+        <v>0</v>
       </c>
       <c r="E31" s="9" t="n">
         <f aca="false">IF(MOD(A31,3)=0,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$23,Paramètres!$C$23,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$22,Paramètres!$C$22,0)),0)</f>
@@ -1951,11 +1951,11 @@
       </c>
       <c r="F31" s="16" t="n">
         <f aca="false">C31+D31+E31</f>
-        <v>2823.25</v>
+        <v>2122</v>
       </c>
       <c r="G31" s="9" t="n">
         <f aca="false">SUM($F$17:F31)</f>
-        <v>31857.25</v>
+        <v>25546</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1972,7 +1972,7 @@
       </c>
       <c r="D32" s="9" t="n">
         <f aca="false">IF(A32&gt;Paramètres!$G$18,$F$11,0)</f>
-        <v>701.25</v>
+        <v>0</v>
       </c>
       <c r="E32" s="9" t="n">
         <f aca="false">IF(MOD(A32,3)=0,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$23,Paramètres!$C$23,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$22,Paramètres!$C$22,0)),0)</f>
@@ -1980,11 +1980,11 @@
       </c>
       <c r="F32" s="16" t="n">
         <f aca="false">C32+D32+E32</f>
-        <v>2568.25</v>
+        <v>1867</v>
       </c>
       <c r="G32" s="9" t="n">
         <f aca="false">SUM($F$17:F32)</f>
-        <v>34425.5</v>
+        <v>27413</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="D33" s="9" t="n">
         <f aca="false">IF(A33&gt;Paramètres!$G$18,$F$11,0)</f>
-        <v>701.25</v>
+        <v>0</v>
       </c>
       <c r="E33" s="9" t="n">
         <f aca="false">IF(MOD(A33,3)=0,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$23,Paramètres!$C$23,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$22,Paramètres!$C$22,0)),0)</f>
@@ -2009,11 +2009,11 @@
       </c>
       <c r="F33" s="16" t="n">
         <f aca="false">C33+D33+E33</f>
-        <v>2568.25</v>
+        <v>1867</v>
       </c>
       <c r="G33" s="9" t="n">
         <f aca="false">SUM($F$17:F33)</f>
-        <v>36993.75</v>
+        <v>29280</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2030,7 +2030,7 @@
       </c>
       <c r="D34" s="9" t="n">
         <f aca="false">IF(A34&gt;Paramètres!$G$18,$F$11,0)</f>
-        <v>701.25</v>
+        <v>0</v>
       </c>
       <c r="E34" s="9" t="n">
         <f aca="false">IF(MOD(A34,3)=0,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$23,Paramètres!$C$23,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$22,Paramètres!$C$22,0)),0)</f>
@@ -2038,11 +2038,11 @@
       </c>
       <c r="F34" s="16" t="n">
         <f aca="false">C34+D34+E34</f>
-        <v>2823.25</v>
+        <v>2122</v>
       </c>
       <c r="G34" s="9" t="n">
         <f aca="false">SUM($F$17:F34)</f>
-        <v>39817</v>
+        <v>31402</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="D35" s="9" t="n">
         <f aca="false">IF(A35&gt;Paramètres!$G$18,$F$11,0)</f>
-        <v>701.25</v>
+        <v>0</v>
       </c>
       <c r="E35" s="9" t="n">
         <f aca="false">IF(MOD(A35,3)=0,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$23,Paramètres!$C$23,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$22,Paramètres!$C$22,0)),0)</f>
@@ -2067,11 +2067,11 @@
       </c>
       <c r="F35" s="16" t="n">
         <f aca="false">C35+D35+E35</f>
-        <v>2568.25</v>
+        <v>1867</v>
       </c>
       <c r="G35" s="9" t="n">
         <f aca="false">SUM($F$17:F35)</f>
-        <v>42385.25</v>
+        <v>33269</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2088,7 +2088,7 @@
       </c>
       <c r="D36" s="9" t="n">
         <f aca="false">IF(A36&gt;Paramètres!$G$18,$F$11,0)</f>
-        <v>701.25</v>
+        <v>0</v>
       </c>
       <c r="E36" s="9" t="n">
         <f aca="false">IF(MOD(A36,3)=0,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$23,Paramètres!$C$23,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$22,Paramètres!$C$22,0)),0)</f>
@@ -2096,11 +2096,11 @@
       </c>
       <c r="F36" s="16" t="n">
         <f aca="false">C36+D36+E36</f>
-        <v>2568.25</v>
+        <v>1867</v>
       </c>
       <c r="G36" s="9" t="n">
         <f aca="false">SUM($F$17:F36)</f>
-        <v>44953.5</v>
+        <v>35136</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2117,7 +2117,7 @@
       </c>
       <c r="D37" s="9" t="n">
         <f aca="false">IF(A37&gt;Paramètres!$G$18,$F$11,0)</f>
-        <v>701.25</v>
+        <v>0</v>
       </c>
       <c r="E37" s="9" t="n">
         <f aca="false">IF(MOD(A37,3)=0,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$23,Paramètres!$C$23,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$22,Paramètres!$C$22,0)),0)</f>
@@ -2125,11 +2125,11 @@
       </c>
       <c r="F37" s="16" t="n">
         <f aca="false">C37+D37+E37</f>
-        <v>2823.25</v>
+        <v>2122</v>
       </c>
       <c r="G37" s="9" t="n">
         <f aca="false">SUM($F$17:F37)</f>
-        <v>47776.75</v>
+        <v>37258</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2146,7 +2146,7 @@
       </c>
       <c r="D38" s="9" t="n">
         <f aca="false">IF(A38&gt;Paramètres!$G$18,$F$11,0)</f>
-        <v>701.25</v>
+        <v>0</v>
       </c>
       <c r="E38" s="9" t="n">
         <f aca="false">IF(MOD(A38,3)=0,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$23,Paramètres!$C$23,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$22,Paramètres!$C$22,0)),0)</f>
@@ -2154,11 +2154,11 @@
       </c>
       <c r="F38" s="16" t="n">
         <f aca="false">C38+D38+E38</f>
-        <v>2568.25</v>
+        <v>1867</v>
       </c>
       <c r="G38" s="9" t="n">
         <f aca="false">SUM($F$17:F38)</f>
-        <v>50345</v>
+        <v>39125</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="D39" s="9" t="n">
         <f aca="false">IF(A39&gt;Paramètres!$G$18,$F$11,0)</f>
-        <v>701.25</v>
+        <v>0</v>
       </c>
       <c r="E39" s="9" t="n">
         <f aca="false">IF(MOD(A39,3)=0,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$23,Paramètres!$C$23,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$22,Paramètres!$C$22,0)),0)</f>
@@ -2183,11 +2183,11 @@
       </c>
       <c r="F39" s="16" t="n">
         <f aca="false">C39+D39+E39</f>
-        <v>2568.25</v>
+        <v>1867</v>
       </c>
       <c r="G39" s="9" t="n">
         <f aca="false">SUM($F$17:F39)</f>
-        <v>52913.25</v>
+        <v>40992</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2204,7 +2204,7 @@
       </c>
       <c r="D40" s="9" t="n">
         <f aca="false">IF(A40&gt;Paramètres!$G$18,$F$11,0)</f>
-        <v>701.25</v>
+        <v>0</v>
       </c>
       <c r="E40" s="9" t="n">
         <f aca="false">IF(MOD(A40,3)=0,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$23,Paramètres!$C$23,IF(3*($C$5+$D$5+$E$5)&gt;=Paramètres!$B$22,Paramètres!$C$22,0)),0)</f>
@@ -2212,11 +2212,11 @@
       </c>
       <c r="F40" s="16" t="n">
         <f aca="false">C40+D40+E40</f>
-        <v>2823.25</v>
+        <v>2122</v>
       </c>
       <c r="G40" s="9" t="n">
         <f aca="false">SUM($F$17:F40)</f>
-        <v>55736.5</v>
+        <v>43114</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2225,7 +2225,7 @@
       </c>
       <c r="F41" s="17" t="n">
         <f aca="false">SUM(F17:F28)</f>
-        <v>23897.5</v>
+        <v>19690</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2234,7 +2234,7 @@
       </c>
       <c r="F42" s="17" t="n">
         <f aca="false">SUM(F29:F40)</f>
-        <v>31839</v>
+        <v>23424</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="F43" s="16" t="n">
         <f aca="false">F42/12</f>
-        <v>2653.25</v>
+        <v>1952</v>
       </c>
     </row>
   </sheetData>
@@ -2386,19 +2386,19 @@
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">-Paramètres!E7*Paramètres!$G$13</f>
-        <v>-34</v>
+        <v>-0</v>
       </c>
       <c r="C9" s="9" t="n">
         <f aca="false">-Paramètres!E8*Paramètres!$G$13</f>
-        <v>-178.5</v>
+        <v>-0</v>
       </c>
       <c r="D9" s="9" t="n">
         <f aca="false">-Paramètres!E9*Paramètres!$G$13</f>
-        <v>-310.25</v>
+        <v>-0</v>
       </c>
       <c r="E9" s="9" t="n">
         <f aca="false">-Paramètres!E10*Paramètres!$G$13</f>
-        <v>-565.25</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2407,19 +2407,19 @@
       </c>
       <c r="B10" s="17" t="n">
         <f aca="false">SUM(B5:B9)</f>
-        <v>460</v>
+        <v>494</v>
       </c>
       <c r="C10" s="17" t="n">
         <f aca="false">SUM(C5:C9)</f>
-        <v>1729.7</v>
+        <v>1908.2</v>
       </c>
       <c r="D10" s="17" t="n">
         <f aca="false">SUM(D5:D9)</f>
-        <v>2836.95</v>
+        <v>3147.2</v>
       </c>
       <c r="E10" s="17" t="n">
         <f aca="false">SUM(E5:E9)</f>
-        <v>4958.95</v>
+        <v>5524.2</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2428,19 +2428,19 @@
       </c>
       <c r="B11" s="20" t="n">
         <f aca="false">IF(B5=0,0,B10/B5)</f>
-        <v>0.485232067510549</v>
+        <v>0.521097046413502</v>
       </c>
       <c r="C11" s="20" t="n">
         <f aca="false">IF(C5=0,0,C10/C5)</f>
-        <v>0.294166666666667</v>
+        <v>0.32452380952381</v>
       </c>
       <c r="D11" s="20" t="n">
         <f aca="false">IF(D5=0,0,D10/D5)</f>
-        <v>0.274898255813954</v>
+        <v>0.304961240310078</v>
       </c>
       <c r="E11" s="20" t="n">
         <f aca="false">IF(E5=0,0,E10/E5)</f>
-        <v>0.263213906581741</v>
+        <v>0.293216560509554</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2449,19 +2449,19 @@
       </c>
       <c r="B12" s="20" t="n">
         <f aca="false">IF(B10-B8-B9=0,0,-(B8+B9)/(B10-B8-B9))</f>
-        <v>0.290123456790123</v>
+        <v>0.237654320987654</v>
       </c>
       <c r="C12" s="20" t="n">
         <f aca="false">IF(C10-C8-C9=0,0,-(C8+C9)/(C10-C8-C9))</f>
-        <v>0.271459860163424</v>
+        <v>0.196276640552607</v>
       </c>
       <c r="D12" s="20" t="n">
         <f aca="false">IF(D10-D8-D9=0,0,-(D8+D9)/(D10-D8-D9))</f>
-        <v>0.277798991904689</v>
+        <v>0.198818797413574</v>
       </c>
       <c r="E12" s="20" t="n">
         <f aca="false">IF(E10-E8-E9=0,0,-(E8+E9)/(E10-E8-E9))</f>
-        <v>0.282372434951232</v>
+        <v>0.200573065902579</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2600,15 +2600,15 @@
       </c>
       <c r="B22" s="9" t="n">
         <f aca="false">B21*B10</f>
-        <v>5520</v>
+        <v>5928</v>
       </c>
       <c r="C22" s="9" t="n">
         <f aca="false">C21*C10</f>
-        <v>41512.8</v>
+        <v>45796.8</v>
       </c>
       <c r="D22" s="9" t="n">
         <f aca="false">D21*D10</f>
-        <v>34043.4</v>
+        <v>37766.4</v>
       </c>
       <c r="E22" s="9" t="n">
         <f aca="false">E21*E10</f>
@@ -2616,7 +2616,7 @@
       </c>
       <c r="F22" s="17" t="n">
         <f aca="false">SUM(B22:E22)</f>
-        <v>81076.2</v>
+        <v>89491.2</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
v53 : secrétaires payées au taux horaire (17 €/h par défaut, négociable) — appli, simulateur, contrat et guide collaborateur
</commit_message>
<xml_diff>
--- a/docs/pack-commercial/commerciaux/SIMULATEUR-COMMISSIONS.xlsx
+++ b/docs/pack-commercial/commerciaux/SIMULATEUR-COMMISSIONS.xlsx
@@ -48,7 +48,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Cf. note de stratégie tarifaire : 65 % du CA secrétariat (l'abonnement appli n'entre pas dans l'assiette).</t>
+          <t xml:space="preserve">17 € / h au démarrage, négociable (cf. note de stratégie tarifaire). Remplace l'ancienne rétrocession de 65 %.</t>
         </r>
       </text>
     </comment>
@@ -134,7 +134,7 @@
     <t xml:space="preserve">Bonus engagement 12 mois</t>
   </si>
   <si>
-    <t xml:space="preserve">Rétrocession secrétaire (65 %)</t>
+    <t xml:space="preserve">Secrétaire / mois (heures × taux)</t>
   </si>
   <si>
     <t xml:space="preserve">Coût technique / mois</t>
@@ -158,7 +158,7 @@
     <t xml:space="preserve">Taux de conservation des garages à M6</t>
   </si>
   <si>
-    <t xml:space="preserve">Rétrocession au collaborateur secrétariat (part du CA secrétariat HT)</t>
+    <t xml:space="preserve">Taux horaire versé à la secrétaire (€ HT / heure de forfait)</t>
   </si>
   <si>
     <t xml:space="preserve">Coût technique par garage et par mois (hébergement, IA, emails)</t>
@@ -191,7 +191,7 @@
     <t xml:space="preserve">Palier 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Source des prix et de la rétrocession : NOTE-STRATEGIE-TARIFAIRE et IDEAFORMA_modele_rentabilite.xlsx (docs/pack-commercial). Commissions : grille apporteurs v1.2 du 25/08/2026 (une prime unique par garage, prime de fidélité supprimée).</t>
+    <t xml:space="preserve">Source des prix et du taux horaire : NOTE-STRATEGIE-TARIFAIRE et IDEAFORMA_modele_rentabilite.xlsx (docs/pack-commercial). Commissions : grille apporteurs v1.2 du 25/08/2026 (une prime unique par garage, prime de fidélité supprimée).</t>
   </si>
   <si>
     <t xml:space="preserve">Ce que gagne le commercial selon son rythme</t>
@@ -278,7 +278,7 @@
     <t xml:space="preserve">Chiffre d'affaires HT (12 mois)</t>
   </si>
   <si>
-    <t xml:space="preserve">Rétrocession secrétariat</t>
+    <t xml:space="preserve">Secrétaire (heures × taux horaire)</t>
   </si>
   <si>
     <t xml:space="preserve">Coûts techniques</t>
@@ -302,7 +302,7 @@
     <t xml:space="preserve">Année 2 et suivantes — par garage</t>
   </si>
   <si>
-    <t xml:space="preserve">Rétrocession secrétariat + coûts techniques</t>
+    <t xml:space="preserve">Secrétaire + coûts techniques</t>
   </si>
   <si>
     <t xml:space="preserve">Marge brute année 2 (aucune commission)</t>
@@ -1061,7 +1061,7 @@
         <v>40</v>
       </c>
       <c r="G7" s="8" t="n">
-        <f aca="false">IF(C7=0,0,(B7-$B$7)*$G$14)</f>
+        <f aca="false">C7*$G$14</f>
         <v>0</v>
       </c>
       <c r="H7" s="9" t="n">
@@ -1089,8 +1089,8 @@
         <v>85</v>
       </c>
       <c r="G8" s="8" t="n">
-        <f aca="false">IF(C8=0,0,(B8-$B$7)*$G$14)</f>
-        <v>267.15</v>
+        <f aca="false">C8*$G$14</f>
+        <v>170</v>
       </c>
       <c r="H8" s="9" t="n">
         <f aca="false">$G$15</f>
@@ -1117,8 +1117,8 @@
         <v>85</v>
       </c>
       <c r="G9" s="8" t="n">
-        <f aca="false">IF(C9=0,0,(B9-$B$7)*$G$14)</f>
-        <v>507.65</v>
+        <f aca="false">C9*$G$14</f>
+        <v>340</v>
       </c>
       <c r="H9" s="9" t="n">
         <f aca="false">$G$15</f>
@@ -1145,8 +1145,8 @@
         <v>85</v>
       </c>
       <c r="G10" s="8" t="n">
-        <f aca="false">IF(C10=0,0,(B10-$B$7)*$G$14)</f>
-        <v>969.15</v>
+        <f aca="false">C10*$G$14</f>
+        <v>680</v>
       </c>
       <c r="H10" s="9" t="n">
         <f aca="false">$G$15</f>
@@ -1180,8 +1180,8 @@
       <c r="D14" s="11"/>
       <c r="E14" s="11"/>
       <c r="F14" s="11"/>
-      <c r="G14" s="12" t="n">
-        <v>0.65</v>
+      <c r="G14" s="6" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2327,15 +2327,15 @@
       </c>
       <c r="C6" s="9" t="n">
         <f aca="false">-Paramètres!G8*12</f>
-        <v>-3205.8</v>
+        <v>-2040</v>
       </c>
       <c r="D6" s="9" t="n">
         <f aca="false">-Paramètres!G9*12</f>
-        <v>-6091.8</v>
+        <v>-4080</v>
       </c>
       <c r="E6" s="9" t="n">
         <f aca="false">-Paramètres!G10*12</f>
-        <v>-11629.8</v>
+        <v>-8160</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2411,15 +2411,15 @@
       </c>
       <c r="C10" s="17" t="n">
         <f aca="false">SUM(C5:C9)</f>
-        <v>1908.2</v>
+        <v>3074</v>
       </c>
       <c r="D10" s="17" t="n">
         <f aca="false">SUM(D5:D9)</f>
-        <v>3147.2</v>
+        <v>5159</v>
       </c>
       <c r="E10" s="17" t="n">
         <f aca="false">SUM(E5:E9)</f>
-        <v>5524.2</v>
+        <v>8994</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2432,15 +2432,15 @@
       </c>
       <c r="C11" s="20" t="n">
         <f aca="false">IF(C5=0,0,C10/C5)</f>
-        <v>0.32452380952381</v>
+        <v>0.522789115646259</v>
       </c>
       <c r="D11" s="20" t="n">
         <f aca="false">IF(D5=0,0,D10/D5)</f>
-        <v>0.304961240310078</v>
+        <v>0.499903100775194</v>
       </c>
       <c r="E11" s="20" t="n">
         <f aca="false">IF(E5=0,0,E10/E5)</f>
-        <v>0.293216560509554</v>
+        <v>0.477388535031847</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2453,15 +2453,15 @@
       </c>
       <c r="C12" s="20" t="n">
         <f aca="false">IF(C10-C8-C9=0,0,-(C8+C9)/(C10-C8-C9))</f>
-        <v>0.196276640552607</v>
+        <v>0.131638418079096</v>
       </c>
       <c r="D12" s="20" t="n">
         <f aca="false">IF(D10-D8-D9=0,0,-(D8+D9)/(D10-D8-D9))</f>
-        <v>0.198818797413574</v>
+        <v>0.131481481481481</v>
       </c>
       <c r="E12" s="20" t="n">
         <f aca="false">IF(E10-E8-E9=0,0,-(E8+E9)/(E10-E8-E9))</f>
-        <v>0.200573065902579</v>
+        <v>0.133526011560694</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2512,15 +2512,15 @@
       </c>
       <c r="C16" s="9" t="n">
         <f aca="false">-(Paramètres!G8+Paramètres!H8)*12</f>
-        <v>-3505.8</v>
+        <v>-2340</v>
       </c>
       <c r="D16" s="9" t="n">
         <f aca="false">-(Paramètres!G9+Paramètres!H9)*12</f>
-        <v>-6391.8</v>
+        <v>-4380</v>
       </c>
       <c r="E16" s="9" t="n">
         <f aca="false">-(Paramètres!G10+Paramètres!H10)*12</f>
-        <v>-11929.8</v>
+        <v>-8460</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2533,15 +2533,15 @@
       </c>
       <c r="C17" s="17" t="n">
         <f aca="false">C15+C16</f>
-        <v>2374.2</v>
+        <v>3540</v>
       </c>
       <c r="D17" s="17" t="n">
         <f aca="false">D15+D16</f>
-        <v>3928.2</v>
+        <v>5940</v>
       </c>
       <c r="E17" s="17" t="n">
         <f aca="false">E15+E16</f>
-        <v>6910.2</v>
+        <v>10380</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2604,11 +2604,11 @@
       </c>
       <c r="C22" s="9" t="n">
         <f aca="false">C21*C10</f>
-        <v>45796.8</v>
+        <v>73776</v>
       </c>
       <c r="D22" s="9" t="n">
         <f aca="false">D21*D10</f>
-        <v>37766.4</v>
+        <v>61908</v>
       </c>
       <c r="E22" s="9" t="n">
         <f aca="false">E21*E10</f>
@@ -2616,7 +2616,7 @@
       </c>
       <c r="F22" s="17" t="n">
         <f aca="false">SUM(B22:E22)</f>
-        <v>89491.2</v>
+        <v>141612</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2629,11 +2629,11 @@
       </c>
       <c r="C23" s="9" t="n">
         <f aca="false">C21*C17*Paramètres!$G$13</f>
-        <v>48433.68</v>
+        <v>72216</v>
       </c>
       <c r="D23" s="9" t="n">
         <f aca="false">D21*D17*Paramètres!$G$13</f>
-        <v>40067.64</v>
+        <v>60588</v>
       </c>
       <c r="E23" s="9" t="n">
         <f aca="false">E21*E17*Paramètres!$G$13</f>
@@ -2641,7 +2641,7 @@
       </c>
       <c r="F23" s="17" t="n">
         <f aca="false">SUM(B23:E23)</f>
-        <v>95110.92</v>
+        <v>139413.6</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Pack v1.4 - guide collaborateur reecrit (contrat v2.1), fiche rentabilite et simulateur en grille v1.3
</commit_message>
<xml_diff>
--- a/docs/pack-commercial/commerciaux/SIMULATEUR-COMMISSIONS.xlsx
+++ b/docs/pack-commercial/commerciaux/SIMULATEUR-COMMISSIONS.xlsx
@@ -128,7 +128,7 @@
     <t xml:space="preserve">Prime de signature</t>
   </si>
   <si>
-    <t xml:space="preserve">Prime de fidélité (0 en v1.2)</t>
+    <t xml:space="preserve">Prime de fidélité (0 depuis la v1.2)</t>
   </si>
   <si>
     <t xml:space="preserve">Bonus engagement 12 mois</t>
@@ -167,7 +167,7 @@
     <t xml:space="preserve">Part des devis signés avec engagement 12 mois</t>
   </si>
   <si>
-    <t xml:space="preserve">Délai avant paiement de la prime de signature (mois après signature)</t>
+    <t xml:space="preserve">Délai avant paiement de la prime (mois après signature) — v1.3 : 1 avec engagement 12 mois, 3 sans engagement</t>
   </si>
   <si>
     <t xml:space="preserve">Délai avant paiement de la prime de fidélité (mois après signature)</t>
@@ -191,13 +191,13 @@
     <t xml:space="preserve">Palier 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Source des prix et du taux horaire : NOTE-STRATEGIE-TARIFAIRE et IDEAFORMA_modele_rentabilite.xlsx (docs/pack-commercial). Commissions : grille apporteurs v1.2 du 25/08/2026 (une prime unique par garage, prime de fidélité supprimée).</t>
+    <t xml:space="preserve">Source des prix et du taux horaire : NOTE-STRATEGIE-TARIFAIRE et IDEAFORMA_modele_rentabilite.xlsx (docs/pack-commercial). Commissions : grille apporteurs v1.3 du 27/08/2026 (une prime unique par garage ; versée dès la 1re mensualité si engagement 12 mois, à la 3e sinon ; reprise si arrêt avant 3 mensualités).</t>
   </si>
   <si>
     <t xml:space="preserve">Ce que gagne le commercial selon son rythme</t>
   </si>
   <si>
-    <t xml:space="preserve">Saisissez vos signatures mensuelles par formule (jaune). Grille v1.2 : une prime par garage signé, acquise à la 2e mensualité payée ; les montants perçus tiennent compte de ce délai (Paramètres).</t>
+    <t xml:space="preserve">Saisissez vos signatures mensuelles par formule (jaune). Grille v1.3 : une prime par garage signé, versée dès la 1re mensualité encaissée avec engagement 12 mois (3e mensualité sans engagement) ; le délai retenu est celui de l'onglet Paramètres (G17).</t>
   </si>
   <si>
     <t xml:space="preserve">Signatures par mois</t>
@@ -1220,7 +1220,7 @@
       <c r="E17" s="11"/>
       <c r="F17" s="11"/>
       <c r="G17" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>